<commit_message>
更新 Init Data, application yml
</commit_message>
<xml_diff>
--- a/modules/app/src/main/java/com/jeesite/modules/app/db/InitAppData.xlsx
+++ b/modules/app/src/main/java/com/jeesite/modules/app/db/InitAppData.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25900" windowHeight="13900" tabRatio="740" activeTab="1"/>
+    <workbookView windowWidth="29900" windowHeight="13060" tabRatio="740" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Module" sheetId="19" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="111">
   <si>
     <t>moduleCode</t>
   </si>
@@ -165,9 +165,6 @@
   </si>
   <si>
     <t>/app/appUpgrade/list</t>
-  </si>
-  <si>
-    <t>IFRAME</t>
   </si>
   <si>
     <t>app:appUpgrade</t>
@@ -423,7 +420,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,13 +452,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -919,148 +909,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1641,11 +1631,9 @@
       <c r="I3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="8"/>
+      <c r="M3" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="P3" s="6" t="s">
         <v>30</v>
@@ -1665,10 +1653,10 @@
         <v>26</v>
       </c>
       <c r="E4" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>30</v>
@@ -1677,13 +1665,11 @@
         <v>31</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="8"/>
+      <c r="M4" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>42</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>30</v>
@@ -1711,21 +1697,21 @@
   <sheetData>
     <row r="1" s="9" customFormat="1" spans="1:3">
       <c r="A1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" ht="17" spans="1:3">
       <c r="A2" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>47</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>30</v>
@@ -1733,10 +1719,10 @@
     </row>
     <row r="3" ht="17" spans="1:3">
       <c r="A3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>30</v>
@@ -1744,10 +1730,10 @@
     </row>
     <row r="4" ht="17" spans="1:3">
       <c r="A4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>30</v>
@@ -1755,10 +1741,10 @@
     </row>
     <row r="5" ht="17" spans="1:3">
       <c r="A5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>53</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>30</v>
@@ -1792,37 +1778,37 @@
   <sheetData>
     <row r="1" s="5" customFormat="1" ht="17" spans="1:11">
       <c r="A1" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>56</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>14</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" ht="17" spans="1:11">
@@ -1830,16 +1816,16 @@
         <v>33</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>35</v>
@@ -1848,7 +1834,7 @@
         <v>30</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" ht="17" spans="1:11">
@@ -1856,25 +1842,25 @@
         <v>33</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>64</v>
-      </c>
       <c r="F3" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" ht="17" spans="1:11">
@@ -1882,25 +1868,25 @@
         <v>33</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" ht="17" spans="1:11">
@@ -1908,16 +1894,16 @@
         <v>33</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>35</v>
@@ -1926,7 +1912,7 @@
         <v>30</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" ht="17" spans="1:11">
@@ -1934,25 +1920,25 @@
         <v>33</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>70</v>
-      </c>
       <c r="F6" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" ht="17" spans="1:11">
@@ -1960,25 +1946,25 @@
         <v>33</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="F7" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" ht="17" spans="1:11">
@@ -1986,13 +1972,13 @@
         <v>33</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>30</v>
@@ -2004,7 +1990,7 @@
         <v>30</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" ht="17" spans="1:11">
@@ -2012,25 +1998,25 @@
         <v>33</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" ht="17" spans="1:11">
@@ -2038,25 +2024,25 @@
         <v>33</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" ht="17" spans="1:11">
@@ -2064,16 +2050,16 @@
         <v>33</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>35</v>
@@ -2082,7 +2068,7 @@
         <v>30</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" ht="17" spans="1:11">
@@ -2090,25 +2076,25 @@
         <v>33</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>79</v>
-      </c>
       <c r="F12" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" ht="17" spans="1:11">
@@ -2116,25 +2102,25 @@
         <v>33</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>81</v>
-      </c>
       <c r="F13" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2160,42 +2146,42 @@
   <sheetData>
     <row r="1" s="3" customFormat="1" spans="1:9">
       <c r="A1" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
         <v>91</v>
-      </c>
-      <c r="C2" t="s">
-        <v>92</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -2235,31 +2221,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2267,28 +2253,28 @@
         <v>100</v>
       </c>
       <c r="B2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" t="s">
         <v>101</v>
-      </c>
-      <c r="C2" t="s">
-        <v>102</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
       </c>
       <c r="E2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" t="s">
         <v>103</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>104</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>105</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>106</v>
-      </c>
-      <c r="I2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2296,28 +2282,28 @@
         <v>200</v>
       </c>
       <c r="B3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" t="s">
         <v>108</v>
-      </c>
-      <c r="C3" t="s">
-        <v>109</v>
       </c>
       <c r="D3" s="1">
         <v>3</v>
       </c>
       <c r="E3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3" t="s">
         <v>110</v>
       </c>
-      <c r="F3" t="s">
-        <v>104</v>
-      </c>
-      <c r="G3" t="s">
-        <v>111</v>
-      </c>
       <c r="H3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I3" t="s">
         <v>106</v>
-      </c>
-      <c r="I3" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>